<commit_message>
Migliorata la resa su stampa
</commit_message>
<xml_diff>
--- a/registro.xlsx
+++ b/registro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\denic\Documents\Repositories\c++\altro\build-EsportazioneFatture-Desktop_Qt_5_15_0_MinGW_32_bit-Debug\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874F921A-C85C-46F8-B43D-BF135C7D5E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B442EA0-750E-4A2C-92D0-52966235BE51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,9 +69,6 @@
     <t>P. IVA</t>
   </si>
   <si>
-    <t>N° operazione</t>
-  </si>
-  <si>
     <t>Spese 22%</t>
   </si>
   <si>
@@ -82,6 +79,9 @@
   </si>
   <si>
     <t>Natura IVA</t>
+  </si>
+  <si>
+    <t>N°op.</t>
   </si>
 </sst>
 </file>
@@ -689,10 +689,10 @@
   <sheetData>
     <row r="1" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>10</v>
@@ -723,14 +723,14 @@
       </c>
       <c r="N1" s="15"/>
       <c r="O1" s="15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P1" s="15"/>
       <c r="Q1" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R1" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="37.5" x14ac:dyDescent="0.25">

</xml_diff>